<commit_message>
fix: atualizar Carabobo 0x0 como RED e enviar relatorio oficial no Telegram
</commit_message>
<xml_diff>
--- a/metodos_aprovados/Sinais_Metodos_Aprovados_2026-08-30.xlsx
+++ b/metodos_aprovados/Sinais_Metodos_Aprovados_2026-08-30.xlsx
@@ -1324,12 +1324,12 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>3x1</t>
+          <t>0x0</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>GREEN</t>
+          <t>RED</t>
         </is>
       </c>
       <c r="H15" t="n">
@@ -1342,10 +1342,10 @@
         <v>200</v>
       </c>
       <c r="K15" t="n">
-        <v>51.07</v>
+        <v>-200</v>
       </c>
       <c r="L15" t="n">
-        <v>0.955</v>
+        <v>-3.74</v>
       </c>
       <c r="M15" t="inlineStr">
         <is>
@@ -1353,7 +1353,7 @@
         </is>
       </c>
       <c r="N15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O15" t="n">
         <v>1.4</v>

</xml_diff>